<commit_message>
Fix: BKU sequence preservation by using physical row indices from Excel sheet instead of non-unique 'No' column values
</commit_message>
<xml_diff>
--- a/BKU 2026.xlsx
+++ b/BKU 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\SistemLaporanBarang\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B7188D-3737-46E6-A791-923A0D80423B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C87F6973-2573-41FB-BFAC-A6C154862862}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="JANUARI" sheetId="21" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">JANUARI!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -6802,7 +6803,7 @@
         <v>51977300</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A85" s="89">
         <v>51</v>
       </c>
@@ -6928,7 +6929,7 @@
       <c r="F91" s="21"/>
       <c r="G91" s="82"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A92" s="89">
         <v>56</v>
       </c>

</xml_diff>